<commit_message>
Correction to flagged entries format.
</commit_message>
<xml_diff>
--- a/results/pretest/20260717_204822_llama8b_instrument_validation_merged/audit/IV_audit_labeling_workbook_v2 - labeled.xlsx
+++ b/results/pretest/20260717_204822_llama8b_instrument_validation_merged/audit/IV_audit_labeling_workbook_v2 - labeled.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\redsk\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\GitHub\llm-conflict-probing\results\pretest\20260717_204822_llama8b_instrument_validation_merged\audit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{408872FA-FC7C-403E-B69C-D6503AD81318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B402A6B5-0440-4DF9-BABF-5210A6684E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7627" uniqueCount="951">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7627" uniqueCount="952">
   <si>
     <t>row_id</t>
   </si>
@@ -7912,6 +7912,9 @@
   </si>
   <si>
     <t>format issue</t>
+  </si>
+  <si>
+    <t>A</t>
   </si>
 </sst>
 </file>
@@ -23912,7 +23915,7 @@
       </c>
       <c r="G622" s="7"/>
       <c r="H622" s="4" t="s">
-        <v>738</v>
+        <v>754</v>
       </c>
       <c r="I622" s="8" t="s">
         <v>950</v>
@@ -23937,7 +23940,7 @@
       </c>
       <c r="G623" s="7"/>
       <c r="H623" s="4" t="s">
-        <v>738</v>
+        <v>754</v>
       </c>
       <c r="I623" s="8" t="s">
         <v>950</v>
@@ -23962,7 +23965,7 @@
       </c>
       <c r="G624" s="7"/>
       <c r="H624" s="4" t="s">
-        <v>738</v>
+        <v>754</v>
       </c>
       <c r="I624" s="8" t="s">
         <v>950</v>
@@ -23987,7 +23990,7 @@
       </c>
       <c r="G625" s="7"/>
       <c r="H625" s="4" t="s">
-        <v>738</v>
+        <v>951</v>
       </c>
       <c r="I625" s="8" t="s">
         <v>950</v>
@@ -24012,7 +24015,7 @@
       </c>
       <c r="G626" s="7"/>
       <c r="H626" s="4" t="s">
-        <v>738</v>
+        <v>754</v>
       </c>
       <c r="I626" s="8" t="s">
         <v>950</v>
@@ -24037,7 +24040,7 @@
       </c>
       <c r="G627" s="7"/>
       <c r="H627" s="4" t="s">
-        <v>738</v>
+        <v>754</v>
       </c>
       <c r="I627" s="8" t="s">
         <v>950</v>
@@ -24062,7 +24065,7 @@
       </c>
       <c r="G628" s="7"/>
       <c r="H628" s="4" t="s">
-        <v>738</v>
+        <v>754</v>
       </c>
       <c r="I628" s="8" t="s">
         <v>950</v>
@@ -24087,7 +24090,7 @@
       </c>
       <c r="G629" s="7"/>
       <c r="H629" s="4" t="s">
-        <v>738</v>
+        <v>951</v>
       </c>
       <c r="I629" s="8" t="s">
         <v>950</v>

</xml_diff>